<commit_message>
결과 파일 업데이트 2026-10-13 05:08
</commit_message>
<xml_diff>
--- a/results/andar_할인율모니터링_20261013.xlsx
+++ b/results/andar_할인율모니터링_20261013.xlsx
@@ -1549,84 +1549,84 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=17437&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=18854&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>EPTCP-03</t>
+          <t>EPTBG-10</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>썬가드 와이드 버킷햇</t>
+          <t>미니 크레센트 듀얼백</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>69,000</t>
+          <t>55,000</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>69,000</t>
+          <t>52,000</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>5%</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>83</t>
+          <t>14</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>4.6</t>
+          <t>4.9</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=18854&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=17437&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>EPTBG-10</t>
+          <t>EPTCP-03</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>미니 크레센트 듀얼백</t>
+          <t>썬가드 와이드 버킷햇</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>55,000</t>
+          <t>69,000</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>52,000</t>
+          <t>69,000</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>83</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>4.6</t>
         </is>
       </c>
     </row>
@@ -1801,84 +1801,84 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=16045&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13862&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>EOTMU-01</t>
+          <t>EOTBG-03</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>스트링 패딩 넥워머</t>
+          <t>데이 앤 트래블 숄더백</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>49,000</t>
+          <t>79,000</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>39,000</t>
+          <t>59,000</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>20%</t>
+          <t>25%</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>135</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>4.6</t>
+          <t>4.9</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13862&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=16045&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>EOTBG-03</t>
+          <t>EOTMU-01</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>데이 앤 트래블 숄더백</t>
+          <t>스트링 패딩 넥워머</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>79,000</t>
+          <t>49,000</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>59,000</t>
+          <t>39,000</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>25%</t>
+          <t>20%</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>135</t>
+          <t>47</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>4.6</t>
         </is>
       </c>
     </row>
@@ -1927,168 +1927,168 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=16031&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=14059&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>EOTGL-02</t>
+          <t>ENTSO-02</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>히트 런 글러브</t>
+          <t>안다르 제트플라이 (우먼즈)</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>29,000</t>
+          <t>139,000</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>29,000</t>
+          <t>95,000</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>32%</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>272</t>
+          <t>1,069</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=17414&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=14059&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>EPTBG-01</t>
+          <t>ENTSO-12</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>에어플라이 프리런 러닝 벨트</t>
+          <t>안다르 제트플라이 (우먼즈)</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>39,000</t>
+          <t>139,000</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>27,000</t>
+          <t>95,000</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>31%</t>
+          <t>32%</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>88</t>
+          <t>1,069</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=14059&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=16031&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>ENTSO-02</t>
+          <t>EOTGL-02</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>안다르 제트플라이 (우먼즈)</t>
+          <t>히트 런 글러브</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>139,000</t>
+          <t>29,000</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>95,000</t>
+          <t>29,000</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>32%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>1,069</t>
+          <t>272</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=14059&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=17414&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>ENTSO-12</t>
+          <t>EPTBG-01</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>안다르 제트플라이 (우먼즈)</t>
+          <t>에어플라이 프리런 러닝 벨트</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>139,000</t>
+          <t>39,000</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>95,000</t>
+          <t>27,000</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>32%</t>
+          <t>31%</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>1,069</t>
+          <t>88</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
@@ -2179,168 +2179,168 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=12487&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=8819&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>ENTBG-18</t>
+          <t>EMTSC-04</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>시티 플로우 빅 숄더백</t>
+          <t>[1&amp;1] 논슬립 서포트 하프 토삭스 (HOLE &amp; SOLID)</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>79,000</t>
+          <t>19,800</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>75,000</t>
+          <t>12,900</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>35%</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>468</t>
+          <t>3,246</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=10478&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=8819&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>ENTBG-05</t>
+          <t>EMTSC-05</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>미니 숄더 앤 크로스백</t>
+          <t>[1&amp;1] 논슬립 서포트 하프 토삭스 (HOLE &amp; SOLID)</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>49,000</t>
+          <t>19,800</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>35,000</t>
+          <t>12,900</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>29%</t>
+          <t>35%</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>5,195</t>
+          <t>3,246</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=8819&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=12487&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>EMTSC-04</t>
+          <t>ENTBG-18</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>[1&amp;1] 논슬립 서포트 하프 토삭스 (HOLE &amp; SOLID)</t>
+          <t>시티 플로우 빅 숄더백</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>19,800</t>
+          <t>79,000</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>12,900</t>
+          <t>75,000</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>35%</t>
+          <t>5%</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>3,246</t>
+          <t>468</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=8819&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=10478&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>EMTSC-05</t>
+          <t>ENTBG-05</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>[1&amp;1] 논슬립 서포트 하프 토삭스 (HOLE &amp; SOLID)</t>
+          <t>미니 숄더 앤 크로스백</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>19,800</t>
+          <t>49,000</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>12,900</t>
+          <t>35,000</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>35%</t>
+          <t>29%</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>3,246</t>
+          <t>5,195</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.9</t>
         </is>
       </c>
     </row>
@@ -2389,121 +2389,121 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=18773&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=17425&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>EPTBG-11</t>
+          <t>EPTSC-06</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>안다르 실버 리유저블백 L</t>
+          <t>필라테스 크루 삭스</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>7,500</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>7,500</t>
+          <t>10,900</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>22%</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>111</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=17425&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=18773&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>EPTSC-06</t>
+          <t>EPTBG-11</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>필라테스 크루 삭스</t>
+          <t>안다르 실버 리유저블백 L</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>7,500</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>10,900</t>
+          <t>7,500</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>22%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>111</t>
+          <t>13</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=16032&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15403&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>EOTCP-05</t>
+          <t>EOTBG-21</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>히트 런 이어플랩 캡</t>
+          <t>데일리 라운드백</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
+          <t>75,000</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
           <t>55,000</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>55,000</t>
-        </is>
-      </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>27%</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>95</t>
+          <t>140</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -2515,37 +2515,37 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15403&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=16868&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>EOTBG-21</t>
+          <t>EPTBG-03</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>데일리 라운드백</t>
+          <t>컴팩트 포켓 크로스백</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>75,000</t>
+          <t>65,000</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>55,000</t>
+          <t>45,000</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>27%</t>
+          <t>31%</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>160</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -2557,37 +2557,37 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=16868&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=16032&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>EPTBG-03</t>
+          <t>EOTCP-05</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>컴팩트 포켓 크로스백</t>
+          <t>히트 런 이어플랩 캡</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>65,000</t>
+          <t>55,000</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>45,000</t>
+          <t>55,000</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>31%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>95</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -2599,17 +2599,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=18767&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=12318&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>EPTBG-06</t>
+          <t>ENTBG-13</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>컴팩트 포켓 스퀘어 크로스백</t>
+          <t>데일리 스퀘어백</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -2619,39 +2619,39 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>65,000</t>
+          <t>49,000</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>6%</t>
+          <t>29%</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>441</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=12318&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=18767&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>ENTBG-13</t>
+          <t>EPTBG-06</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>데일리 스퀘어백</t>
+          <t>컴팩트 포켓 스퀘어 크로스백</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -2661,59 +2661,59 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>49,000</t>
+          <t>65,000</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>29%</t>
+          <t>6%</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>441</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13853&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15629&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>EOTBG-12</t>
+          <t>EOTBG-23</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>프리런 벨크로 러닝 벨트</t>
+          <t>안다르 실버 리유저블백 M</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>35,000</t>
+          <t>6,500</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>29,000</t>
+          <t>6,500</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>17%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>256</t>
+          <t>410</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -2725,84 +2725,84 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15350&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13853&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>EOTSC-09</t>
+          <t>EOTBG-12</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>[1&amp;1] 컴프레션 러닝 니삭스</t>
+          <t>프리런 벨크로 러닝 벨트</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>29,800</t>
+          <t>35,000</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>21,900</t>
+          <t>29,000</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>27%</t>
+          <t>17%</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>725</t>
+          <t>256</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15629&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15350&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>EOTBG-23</t>
+          <t>EOTSC-09</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>안다르 실버 리유저블백 M</t>
+          <t>[1&amp;1] 컴프레션 러닝 니삭스</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>6,500</t>
+          <t>29,800</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>6,500</t>
+          <t>21,900</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>27%</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>410</t>
+          <t>725</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
@@ -2851,205 +2851,205 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=18772&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=8769&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>EPTFR-01</t>
+          <t>EMTSV-02</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>폼롤러</t>
+          <t>[1ea] 서포트 발목 보호대</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>59,000</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>55,000</t>
+          <t>9,900</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>7%</t>
+          <t>29%</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>742</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=18772&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13409&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>EPTFR-02</t>
+          <t>EOTBG-10</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>폼롤러</t>
+          <t>에어플라이 투웨이 프리런 백 3.0</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>59,000</t>
+          <t>35,000</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>55,000</t>
+          <t>32,000</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>7%</t>
+          <t>9%</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1,171</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>3.0</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=8769&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=18772&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>EMTSV-02</t>
+          <t>EPTFR-01</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>[1ea] 서포트 발목 보호대</t>
+          <t>폼롤러</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>59,000</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>9,900</t>
+          <t>55,000</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>29%</t>
+          <t>7%</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>742</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>5.0</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13409&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=18772&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>EOTBG-10</t>
+          <t>EPTFR-02</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>에어플라이 투웨이 프리런 백 3.0</t>
+          <t>폼롤러</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>35,000</t>
+          <t>59,000</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>32,000</t>
+          <t>55,000</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>9%</t>
+          <t>7%</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>1,171</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>5.0</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13408&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=17423&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>EOTSC-01</t>
+          <t>EPTSC-04</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>프레시 필드 니삭스</t>
+          <t>필라테스 토삭스</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>14,900</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>14,900</t>
+          <t>10,900</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>22%</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>307</t>
+          <t>113</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
@@ -3103,37 +3103,37 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=18761&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13408&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>EPTRB-02</t>
+          <t>EOTSC-01</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>9스텝 스트레칭 밴드</t>
+          <t>프레시 필드 니삭스</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>15,900</t>
+          <t>14,900</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>14,900</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>13%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>307</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
@@ -3145,37 +3145,37 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=17423&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=18761&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>EPTSC-04</t>
+          <t>EPTRB-02</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>필라테스 토삭스</t>
+          <t>9스텝 스트레칭 밴드</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
+          <t>15,900</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
           <t>13,900</t>
         </is>
       </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>10,900</t>
-        </is>
-      </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>22%</t>
+          <t>13%</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>113</t>
+          <t>18</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
@@ -3187,27 +3187,27 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=6952&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15408&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>EJFST-02</t>
+          <t>EOTSC-14</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>릴렉스 요가링</t>
+          <t>맨즈 논슬립 풀 토삭스</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>5,900</t>
+          <t>11,900</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>3,900</t>
+          <t>7,900</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -3217,49 +3217,49 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>6,654</t>
+          <t>115</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.6</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13604&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=6952&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>EOTSV-01</t>
+          <t>EJFST-02</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>[2ea] 하이 서포트 무릎 보호대</t>
+          <t>릴렉스 요가링</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>29,800</t>
+          <t>5,900</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>19,900</t>
+          <t>3,900</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>33%</t>
+          <t>34%</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>742</t>
+          <t>6,654</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
@@ -3271,121 +3271,121 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15408&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13604&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>EOTSC-14</t>
+          <t>EOTSV-01</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>맨즈 논슬립 풀 토삭스</t>
+          <t>[2ea] 하이 서포트 무릎 보호대</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>11,900</t>
+          <t>29,800</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>7,900</t>
+          <t>19,900</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>34%</t>
+          <t>33%</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>115</t>
+          <t>742</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>4.6</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15143&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=10948&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>EOTBG-17</t>
+          <t>ENTSC-20</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>3 in 1 캐리온 더플백</t>
+          <t>시그니처 로고 크루 삭스</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>109,000</t>
+          <t>7,900</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>85,000</t>
+          <t>5,900</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>22%</t>
+          <t>25%</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>612</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.9</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=10948&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=11962&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>ENTSC-20</t>
+          <t>ENTMT-01</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>시그니처 로고 크루 삭스</t>
+          <t>레스트 인 마블 요가매트 (4mm)</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>7,900</t>
+          <t>49,000</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>5,900</t>
+          <t>45,000</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>25%</t>
+          <t>8%</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>612</t>
+          <t>277</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
@@ -3397,37 +3397,37 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15371&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15143&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>EOTBG-15</t>
+          <t>EOTBG-17</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>폴더블 짐백 2.0</t>
+          <t>3 in 1 캐리온 더플백</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>59,000</t>
+          <t>109,000</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>45,000</t>
+          <t>85,000</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>24%</t>
+          <t>22%</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>48</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
@@ -3523,121 +3523,121 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=18765&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15371&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>EPTSC-11</t>
+          <t>EOTBG-15</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>데일리 쿠션 크루 삭스</t>
+          <t>폴더블 짐백 2.0</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>8,900</t>
+          <t>59,000</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>7,900</t>
+          <t>45,000</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>11%</t>
+          <t>24%</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>60</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=11962&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=18765&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>ENTMT-01</t>
+          <t>EPTSC-11</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>레스트 인 마블 요가매트 (4mm)</t>
+          <t>데일리 쿠션 크루 삭스</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>49,000</t>
+          <t>8,900</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>45,000</t>
+          <t>7,900</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>8%</t>
+          <t>11%</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>277</t>
+          <t>21</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>5.0</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=16844&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=9996&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>EPTET-02</t>
+          <t>EMTSC-27</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>언더웨어 세탁망</t>
+          <t>올라운드 오버 니삭스</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>9,900</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>9,900</t>
+          <t>10,900</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>22%</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>319</t>
+          <t>299</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
@@ -3649,79 +3649,79 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=16631&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13859&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>EPTSV-03</t>
+          <t>ENTSO-12</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>컴프레션 카프 슬리브 (종아리 보호대)</t>
+          <t>안다르 제트플라이 (맨즈)</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>14,900</t>
+          <t>139,000</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>11,900</t>
+          <t>95,000</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>20%</t>
+          <t>32%</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>275</t>
+          <t>700</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=9996&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=16844&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>EMTSC-27</t>
+          <t>EPTET-02</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>올라운드 오버 니삭스</t>
+          <t>언더웨어 세탁망</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>9,900</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>10,900</t>
+          <t>9,900</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>22%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>299</t>
+          <t>319</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
@@ -3733,42 +3733,42 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13859&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=16631&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>ENTSO-12</t>
+          <t>EPTSV-03</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>안다르 제트플라이 (맨즈)</t>
+          <t>컴프레션 카프 슬리브 (종아리 보호대)</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>139,000</t>
+          <t>14,900</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>95,000</t>
+          <t>11,900</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>32%</t>
+          <t>20%</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>700</t>
+          <t>275</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
@@ -3817,84 +3817,84 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13851&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15370&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>EOTCP-03</t>
+          <t>EOTBG-14</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>쿨 라운드 볼캡</t>
+          <t>폴더블 캐리백 2.0</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>45,000</t>
+          <t>69,000</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>45,000</t>
+          <t>55,000</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>20%</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>110</t>
+          <t>94</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.9</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15370&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13851&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>EOTBG-14</t>
+          <t>EOTCP-03</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>폴더블 캐리백 2.0</t>
+          <t>쿨 라운드 볼캡</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>69,000</t>
+          <t>45,000</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>55,000</t>
+          <t>45,000</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>20%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>94</t>
+          <t>110</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
@@ -4027,37 +4027,37 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=8578&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15153&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>EMTSC-01</t>
+          <t>EOTSC-13</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>링글 크루 삭스</t>
+          <t>테이핑 러닝 삭스</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
+          <t>13,900</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
           <t>7,900</t>
         </is>
       </c>
-      <c r="E87" t="inlineStr">
-        <is>
-          <t>4,900</t>
-        </is>
-      </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>38%</t>
+          <t>43%</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>1,352</t>
+          <t>306</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
@@ -4069,84 +4069,84 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13410&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=11458&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>EOTSC-09</t>
+          <t>ENTSC-13</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>컴프레션 러닝 니삭스</t>
+          <t>논슬립 퍼포먼스 크루삭스</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>14,900</t>
+          <t>11,900</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>12,900</t>
+          <t>8,900</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>13%</t>
+          <t>25%</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>363</t>
+          <t>677</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=8621&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13410&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>EMTSV-06</t>
+          <t>EOTSC-09</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>에어쿨링 손목 보호대</t>
+          <t>컴프레션 러닝 니삭스</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>15,900</t>
+          <t>14,900</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>11,900</t>
+          <t>12,900</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>25%</t>
+          <t>13%</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>1,116</t>
+          <t>363</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.9</t>
         </is>
       </c>
     </row>
@@ -4195,37 +4195,37 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15153&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13404&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>EOTSC-13</t>
+          <t>EOTGL-01</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>테이핑 러닝 삭스</t>
+          <t>짐 글러브 2.0</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>25,000</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>7,900</t>
+          <t>21,000</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>43%</t>
+          <t>16%</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>306</t>
+          <t>300</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
@@ -4237,121 +4237,121 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=11458&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=8578&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>ENTSC-13</t>
+          <t>EMTSC-01</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>논슬립 퍼포먼스 크루삭스</t>
+          <t>링글 크루 삭스</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>11,900</t>
+          <t>7,900</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>8,900</t>
+          <t>4,900</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>25%</t>
+          <t>38%</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>677</t>
+          <t>1,352</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13404&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=8621&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>EOTGL-01</t>
+          <t>EMTSV-06</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>짐 글러브 2.0</t>
+          <t>에어쿨링 손목 보호대</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>25,000</t>
+          <t>15,900</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>21,000</t>
+          <t>11,900</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>16%</t>
+          <t>25%</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>300</t>
+          <t>1,117</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=5837&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=9989&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>EJFMB-03</t>
+          <t>EMTET-02</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>릴렉스 짐볼 65cm</t>
+          <t>소프트 쿠셔닝 훌라후프</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>19,000</t>
+          <t>25,000</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>19,000</t>
+          <t>15,000</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>40%</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>2,133</t>
+          <t>665</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
@@ -4405,37 +4405,37 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=9989&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=5837&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>EMTET-02</t>
+          <t>EJFMB-03</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>소프트 쿠셔닝 훌라후프</t>
+          <t>릴렉스 짐볼 65cm</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>25,000</t>
+          <t>19,000</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>15,000</t>
+          <t>19,000</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>40%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>665</t>
+          <t>2,133</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
@@ -4447,37 +4447,37 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=18759&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=10953&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>EPTMB-01</t>
+          <t>ENTSC-07</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>마사지 싱글볼</t>
+          <t>[3 SET] 에어컴피 크루 삭스</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>11,900</t>
+          <t>51,000</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>10,900</t>
+          <t>29,000</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>8%</t>
+          <t>43%</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>572</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
@@ -4489,252 +4489,252 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=10953&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=11459&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>ENTSC-07</t>
+          <t>ENTSC-14</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>[3 SET] 에어컴피 크루 삭스</t>
+          <t>논슬립 퍼포먼스 니삭스</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>51,000</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>29,000</t>
+          <t>9,900</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>43%</t>
+          <t>29%</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>572</t>
+          <t>758</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=11459&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=18759&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>ENTSC-14</t>
+          <t>EPTMB-01</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>논슬립 퍼포먼스 니삭스</t>
+          <t>마사지 싱글볼</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>11,900</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>9,900</t>
+          <t>10,900</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>29%</t>
+          <t>8%</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>758</t>
+          <t>19</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.9</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=18760&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15377&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>EPTMB-02</t>
+          <t>EOTGL-04</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>마사지 듀얼볼</t>
+          <t>논슬립 스킨 요기 글러브</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>15,900</t>
+          <t>10,900</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>7,900</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>13%</t>
+          <t>28%</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>206</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>4.5</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15377&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=18760&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>EOTGL-04</t>
+          <t>EPTMB-02</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>논슬립 스킨 요기 글러브</t>
+          <t>마사지 듀얼볼</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>10,900</t>
+          <t>15,900</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>7,900</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>28%</t>
+          <t>13%</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>206</t>
+          <t>13</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>4.5</t>
+          <t>4.9</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=10188&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15431&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>EMTRB-01</t>
+          <t>ENTSC-19</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>서포트 힙 밴드</t>
+          <t>[1&amp;1] 맨즈 논슬립 토삭스</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>8,900</t>
+          <t>23,800</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>6,900</t>
+          <t>14,900</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>22%</t>
+          <t>37%</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>1,394</t>
+          <t>334</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=10188&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15431&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>EMTRB-02</t>
+          <t>EOTSC-14</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>서포트 힙 밴드</t>
+          <t>[1&amp;1] 맨즈 논슬립 토삭스</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>8,900</t>
+          <t>23,800</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>6,900</t>
+          <t>14,900</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>22%</t>
+          <t>37%</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>1,394</t>
+          <t>334</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
@@ -4746,7 +4746,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>EMTRB-03</t>
+          <t>EMTRB-01</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -4783,79 +4783,79 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=6661&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=10188&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>EKPMB-01</t>
+          <t>EMTRB-02</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>릴렉스 웨이트볼 0.5kg</t>
+          <t>서포트 힙 밴드</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
+          <t>8,900</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
           <t>6,900</t>
         </is>
       </c>
-      <c r="E105" t="inlineStr">
-        <is>
-          <t>6,500</t>
-        </is>
-      </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>6%</t>
+          <t>22%</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>711</t>
+          <t>1,394</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=16637&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=10188&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>EPTFB-02</t>
+          <t>EMTRB-03</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>퍼포먼스 심리스 손목밴드</t>
+          <t>서포트 힙 밴드</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
+          <t>8,900</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
           <t>6,900</t>
         </is>
       </c>
-      <c r="E106" t="inlineStr">
-        <is>
-          <t>5,900</t>
-        </is>
-      </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>14%</t>
+          <t>22%</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>300</t>
+          <t>1,394</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
@@ -4867,126 +4867,126 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=14561&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=6661&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>EOTBG-05</t>
+          <t>EKPMB-01</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>메쉬 포켓 비치백</t>
+          <t>릴렉스 웨이트볼 0.5kg</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>49,000</t>
+          <t>6,900</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>19,000</t>
+          <t>6,500</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>61%</t>
+          <t>6%</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>711</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15431&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=14561&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>ENTSC-19</t>
+          <t>EOTBG-05</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>[1&amp;1] 맨즈 논슬립 토삭스</t>
+          <t>메쉬 포켓 비치백</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>23,800</t>
+          <t>49,000</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>14,900</t>
+          <t>19,000</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>37%</t>
+          <t>61%</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>334</t>
+          <t>69</t>
         </is>
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.9</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15431&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=16637&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>EOTSC-14</t>
+          <t>EPTFB-02</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>[1&amp;1] 맨즈 논슬립 토삭스</t>
+          <t>퍼포먼스 심리스 손목밴드</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>23,800</t>
+          <t>6,900</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>14,900</t>
+          <t>5,900</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>37%</t>
+          <t>14%</t>
         </is>
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>334</t>
+          <t>300</t>
         </is>
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
@@ -5035,185 +5035,185 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=12765&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=11457&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>ENTBG-16</t>
+          <t>ENTSC-12</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>라이트 패딩 쇼퍼백</t>
+          <t>논슬립 퍼포먼스 토삭스</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>69,000</t>
+          <t>12,900</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>69,000</t>
+          <t>8,900</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>31%</t>
         </is>
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>635</t>
+          <t>4,138</t>
         </is>
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=11457&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=12765&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>ENTSC-12</t>
+          <t>ENTBG-16</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>논슬립 퍼포먼스 토삭스</t>
+          <t>라이트 패딩 쇼퍼백</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>12,900</t>
+          <t>69,000</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>8,900</t>
+          <t>69,000</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>31%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>4,138</t>
+          <t>635</t>
         </is>
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13407&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15867&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>EOTSV-03</t>
+          <t>EOTSC-18</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>[1ea] 서포트 허리 보호대</t>
+          <t>[1&amp;1] 올데이 기모 삭스</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>34,000</t>
+          <t>21,800</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>25,000</t>
+          <t>14,900</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>26%</t>
+          <t>32%</t>
         </is>
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>203</t>
+          <t>228</t>
         </is>
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15867&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13407&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>EOTSC-18</t>
+          <t>EOTSV-03</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>[1&amp;1] 올데이 기모 삭스</t>
+          <t>[1ea] 서포트 허리 보호대</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>21,800</t>
+          <t>34,000</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>14,900</t>
+          <t>25,000</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>32%</t>
+          <t>26%</t>
         </is>
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>228</t>
+          <t>203</t>
         </is>
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15733&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=8727&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>EOTSC-19</t>
+          <t>EMTSC-04</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>레그 숏 워머</t>
+          <t>논슬립 서포트 하프 토삭스 (HOLE)</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -5223,22 +5223,22 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>6,900</t>
+          <t>7,900</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>37%</t>
+          <t>28%</t>
         </is>
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>651</t>
         </is>
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
@@ -5581,27 +5581,27 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=12096&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=12793&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>ENTET-02</t>
+          <t>ENTMU-01</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>릴렉스 소프트 웨이트바 2kg</t>
+          <t>소프트 니트 머플러</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>39,000</t>
+          <t>19,900</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>39,000</t>
+          <t>19,900</t>
         </is>
       </c>
       <c r="F124" t="inlineStr">
@@ -5611,91 +5611,91 @@
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>77</t>
+          <t>480</t>
         </is>
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=12793&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=11130&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>ENTMU-01</t>
+          <t>ENTSV-01</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>소프트 니트 머플러</t>
+          <t>[1&amp;1] 3D 쿨링 팔토시</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
+          <t>29,800</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
           <t>19,900</t>
         </is>
       </c>
-      <c r="E125" t="inlineStr">
-        <is>
-          <t>19,900</t>
-        </is>
-      </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>33%</t>
         </is>
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>566</t>
         </is>
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=11130&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=12096&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>ENTSV-01</t>
+          <t>ENTET-02</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>[1&amp;1] 3D 쿨링 팔토시</t>
+          <t>릴렉스 소프트 웨이트바 2kg</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>29,800</t>
+          <t>39,000</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>19,900</t>
+          <t>39,000</t>
         </is>
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>33%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>566</t>
+          <t>77</t>
         </is>
       </c>
       <c r="H126" t="inlineStr">
@@ -5833,37 +5833,37 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=8727&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=10191&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>EMTSC-04</t>
+          <t>EMTSC-26</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>논슬립 서포트 하프 토삭스 (HOLE)</t>
+          <t>[1&amp;1] 램스울 크루 삭스</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>10,900</t>
+          <t>19,800</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>7,900</t>
+          <t>17,900</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>28%</t>
+          <t>10%</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>651</t>
+          <t>882</t>
         </is>
       </c>
       <c r="H130" t="inlineStr">
@@ -5875,121 +5875,121 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=10191&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=8836&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>EMTSC-26</t>
+          <t>EMTSV-01</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>[1&amp;1] 램스울 크루 삭스</t>
+          <t>[2ea] 서포트 팔꿈치 보호대</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>19,800</t>
+          <t>27,800</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>17,900</t>
+          <t>16,900</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>10%</t>
+          <t>39%</t>
         </is>
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>882</t>
+          <t>605</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15376&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=9612&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>EOTSC-17</t>
+          <t>EMTSC-28</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>논슬립 스킨 토삭스</t>
+          <t>[1&amp;1] 리브드 셔링 루즈 삭스</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>12,900</t>
+          <t>21,800</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>8,900</t>
+          <t>17,900</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>31%</t>
+          <t>18%</t>
         </is>
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>92</t>
+          <t>396</t>
         </is>
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=8836&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15376&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>EMTSV-01</t>
+          <t>EOTSC-17</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>[2ea] 서포트 팔꿈치 보호대</t>
+          <t>논슬립 스킨 토삭스</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>27,800</t>
+          <t>12,900</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>16,900</t>
+          <t>8,900</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>39%</t>
+          <t>31%</t>
         </is>
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>605</t>
+          <t>92</t>
         </is>
       </c>
       <c r="H133" t="inlineStr">
@@ -6001,84 +6001,84 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=6662&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15733&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>EKPMB-02</t>
+          <t>EOTSC-19</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>릴렉스 미니 짐볼</t>
+          <t>레그 숏 워머</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>13,000</t>
+          <t>10,900</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>9,900</t>
+          <t>6,900</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>24%</t>
+          <t>37%</t>
         </is>
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>1,247</t>
+          <t>18</t>
         </is>
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>4.6</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=9612&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=6662&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>EMTSC-28</t>
+          <t>EKPMB-02</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>[1&amp;1] 리브드 셔링 루즈 삭스</t>
+          <t>릴렉스 미니 짐볼</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>21,800</t>
+          <t>13,000</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>17,900</t>
+          <t>9,900</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>18%</t>
+          <t>24%</t>
         </is>
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>396</t>
+          <t>1,247</t>
         </is>
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.6</t>
         </is>
       </c>
     </row>
@@ -6169,37 +6169,37 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13405&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13806&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>EOTSV-01</t>
+          <t>EOTSC-05</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>[1ea] 하이 서포트 무릎 보호대</t>
+          <t>올데이 수피마 앵클 삭스</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>14,900</t>
+          <t>6,900</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>10,900</t>
+          <t>4,900</t>
         </is>
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>27%</t>
+          <t>29%</t>
         </is>
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>742</t>
+          <t>483</t>
         </is>
       </c>
       <c r="H138" t="inlineStr">
@@ -6211,37 +6211,37 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13806&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13405&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>EOTSC-05</t>
+          <t>EOTSV-01</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>올데이 수피마 앵클 삭스</t>
+          <t>[1ea] 하이 서포트 무릎 보호대</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>6,900</t>
+          <t>14,900</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>4,900</t>
+          <t>10,900</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>29%</t>
+          <t>27%</t>
         </is>
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>483</t>
+          <t>742</t>
         </is>
       </c>
       <c r="H139" t="inlineStr">
@@ -6505,27 +6505,27 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=9988&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13842&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>EMTSC-26</t>
+          <t>EOTBG-04</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>램스울 크루 삭스</t>
+          <t>데님 포켓 숄더백</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>9,900</t>
+          <t>59,000</t>
         </is>
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>9,900</t>
+          <t>59,000</t>
         </is>
       </c>
       <c r="F146" t="inlineStr">
@@ -6535,29 +6535,29 @@
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>366</t>
+          <t>39</t>
         </is>
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13842&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=9023&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>EOTBG-04</t>
+          <t>EMTBG-03</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>데님 포켓 숄더백</t>
+          <t>숄더 앤 크로스백</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
@@ -6577,39 +6577,39 @@
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>39</t>
+          <t>8,334</t>
         </is>
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.9</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=9023&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15734&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>EMTBG-03</t>
+          <t>EOTSC-20</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>숄더 앤 크로스백</t>
+          <t>레그 미들 워머</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>59,000</t>
+          <t>12,900</t>
         </is>
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>59,000</t>
+          <t>12,900</t>
         </is>
       </c>
       <c r="F148" t="inlineStr">
@@ -6619,7 +6619,7 @@
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>8,333</t>
+          <t>48</t>
         </is>
       </c>
       <c r="H148" t="inlineStr">
@@ -6673,27 +6673,27 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15734&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=9988&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>EOTSC-20</t>
+          <t>EMTSC-26</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>레그 미들 워머</t>
+          <t>램스울 크루 삭스</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>12,900</t>
+          <t>9,900</t>
         </is>
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>12,900</t>
+          <t>9,900</t>
         </is>
       </c>
       <c r="F150" t="inlineStr">
@@ -6703,7 +6703,7 @@
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>366</t>
         </is>
       </c>
       <c r="H150" t="inlineStr">
@@ -6799,69 +6799,69 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=14085&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=6665&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>EOTSV-04</t>
+          <t>EKPRB-05</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>프리런 라이트 러닝 밴드</t>
+          <t>릴렉스 4레벨 힙 밴드</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>32,000</t>
+          <t>21,900</t>
         </is>
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>22,000</t>
+          <t>21,900</t>
         </is>
       </c>
       <c r="F153" t="inlineStr">
         <is>
-          <t>31%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G153" t="inlineStr">
         <is>
-          <t>130</t>
+          <t>530</t>
         </is>
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>4.2</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=6665&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13831&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>EKPRB-05</t>
+          <t>EOTCP-02</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>릴렉스 4레벨 힙 밴드</t>
+          <t>데님 로고 볼캡</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>21,900</t>
+          <t>39,000</t>
         </is>
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>21,900</t>
+          <t>39,000</t>
         </is>
       </c>
       <c r="F154" t="inlineStr">
@@ -6871,7 +6871,7 @@
       </c>
       <c r="G154" t="inlineStr">
         <is>
-          <t>530</t>
+          <t>26</t>
         </is>
       </c>
       <c r="H154" t="inlineStr">
@@ -6883,79 +6883,79 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=9993&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=17387&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>EMTSC-29</t>
+          <t>EPTSC-08</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>니트 루즈 삭스</t>
+          <t>맨즈 필라테스 크루 삭스</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>9,900</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>7,900</t>
+          <t>10,900</t>
         </is>
       </c>
       <c r="F155" t="inlineStr">
         <is>
-          <t>20%</t>
+          <t>22%</t>
         </is>
       </c>
       <c r="G155" t="inlineStr">
         <is>
-          <t>518</t>
+          <t>4</t>
         </is>
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>5.0</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13831&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=9993&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>EOTCP-02</t>
+          <t>EMTSC-29</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>데님 로고 볼캡</t>
+          <t>니트 루즈 삭스</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>39,000</t>
+          <t>9,900</t>
         </is>
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>39,000</t>
+          <t>7,900</t>
         </is>
       </c>
       <c r="F156" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>20%</t>
         </is>
       </c>
       <c r="G156" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>518</t>
         </is>
       </c>
       <c r="H156" t="inlineStr">
@@ -6967,126 +6967,126 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=17387&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=14085&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>EPTSC-08</t>
+          <t>EOTSV-04</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>맨즈 필라테스 크루 삭스</t>
+          <t>프리런 라이트 러닝 밴드</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>32,000</t>
         </is>
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>10,900</t>
+          <t>22,000</t>
         </is>
       </c>
       <c r="F157" t="inlineStr">
         <is>
-          <t>22%</t>
+          <t>31%</t>
         </is>
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>130</t>
         </is>
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>4.2</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=6666&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=11061&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>EKPET-01</t>
+          <t>ENTSV-01</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>릴렉스 소프트 웨이트바 1kg</t>
+          <t>3D 쿨링 팔토시</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>20,900</t>
+          <t>14,900</t>
         </is>
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>19,000</t>
+          <t>10,900</t>
         </is>
       </c>
       <c r="F158" t="inlineStr">
         <is>
-          <t>9%</t>
+          <t>27%</t>
         </is>
       </c>
       <c r="G158" t="inlineStr">
         <is>
-          <t>603</t>
+          <t>566</t>
         </is>
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=11061&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=6666&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>ENTSV-01</t>
+          <t>EKPET-01</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>3D 쿨링 팔토시</t>
+          <t>릴렉스 소프트 웨이트바 1kg</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>14,900</t>
+          <t>20,900</t>
         </is>
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>10,900</t>
+          <t>19,000</t>
         </is>
       </c>
       <c r="F159" t="inlineStr">
         <is>
-          <t>27%</t>
+          <t>9%</t>
         </is>
       </c>
       <c r="G159" t="inlineStr">
         <is>
-          <t>566</t>
+          <t>603</t>
         </is>
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
@@ -7219,84 +7219,84 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=17386&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13805&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>EPTSC-07</t>
+          <t>EOTSC-04</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>맨즈 필라테스 앵클 삭스</t>
+          <t>올데이 수피마 스니커즈 삭스</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>5,900</t>
         </is>
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>10,900</t>
+          <t>4,500</t>
         </is>
       </c>
       <c r="F163" t="inlineStr">
         <is>
-          <t>22%</t>
+          <t>24%</t>
         </is>
       </c>
       <c r="G163" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>445</t>
         </is>
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13805&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=17386&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>EOTSC-04</t>
+          <t>EPTSC-07</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>올데이 수피마 스니커즈 삭스</t>
+          <t>맨즈 필라테스 앵클 삭스</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>5,900</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>4,500</t>
+          <t>10,900</t>
         </is>
       </c>
       <c r="F164" t="inlineStr">
         <is>
-          <t>24%</t>
+          <t>22%</t>
         </is>
       </c>
       <c r="G164" t="inlineStr">
         <is>
-          <t>445</t>
+          <t>9</t>
         </is>
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>5.0</t>
         </is>
       </c>
     </row>
@@ -7597,166 +7597,166 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=17842&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=19330&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>EPTSC-03</t>
+          <t>EPTSC-12</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>데일리 루즈 삭스</t>
+          <t>소프트 니트 기모 오버 니삭스</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>11,900</t>
+          <t>17,900</t>
         </is>
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>8,900</t>
+          <t>17,900</t>
         </is>
       </c>
       <c r="F172" t="inlineStr">
         <is>
-          <t>25%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G172" t="inlineStr">
         <is>
-          <t>32</t>
-        </is>
-      </c>
-      <c r="H172" t="inlineStr">
-        <is>
-          <t>4.8</t>
-        </is>
-      </c>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H172" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=17440&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=17842&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>EPTET-03</t>
+          <t>EPTSC-03</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>안다르 3단 양우산</t>
+          <t>데일리 루즈 삭스</t>
         </is>
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>29,000</t>
+          <t>11,900</t>
         </is>
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>29,000</t>
+          <t>8,900</t>
         </is>
       </c>
       <c r="F173" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>25%</t>
         </is>
       </c>
       <c r="G173" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>32</t>
         </is>
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>4.4</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=11092&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=17440&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>ENTSC-05</t>
+          <t>EPTET-03</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>에어프레시 크루 삭스</t>
+          <t>안다르 3단 양우산</t>
         </is>
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>17,000</t>
+          <t>29,000</t>
         </is>
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t>12,000</t>
+          <t>29,000</t>
         </is>
       </c>
       <c r="F174" t="inlineStr">
         <is>
-          <t>29%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G174" t="inlineStr">
         <is>
-          <t>575</t>
+          <t>40</t>
         </is>
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.4</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=19330&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=11092&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>EPTSC-12</t>
+          <t>ENTSC-05</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>소프트 니트 기모 오버 니삭스</t>
+          <t>에어프레시 크루 삭스</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>17,900</t>
+          <t>17,000</t>
         </is>
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>17,900</t>
+          <t>12,000</t>
         </is>
       </c>
       <c r="F175" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>29%</t>
         </is>
       </c>
       <c r="G175" t="inlineStr">
         <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H175" t="inlineStr"/>
+          <t>575</t>
+        </is>
+      </c>
+      <c r="H175" t="inlineStr">
+        <is>
+          <t>4.8</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>